<commit_message>
DCM template parameter xlsx updated so the large 'adipose' tissue compartment is now entered as 'rob', to facilitate use of univ_blood() testing.
</commit_message>
<xml_diff>
--- a/Inputs/DCM_template_parameters_Model.xlsx
+++ b/Inputs/DCM_template_parameters_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/bernstein_amanda_epa_gov/Documents/Documents/PKWG_models/pbpk_template_project/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="527" documentId="8_{D031EE4F-1494-41E6-A9B6-B336235EFD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA803394-073A-4194-9F7A-6FF5820C79BF}"/>
+  <xr:revisionPtr revIDLastSave="539" documentId="8_{D031EE4F-1494-41E6-A9B6-B336235EFD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3697E202-808F-42B4-8F54-B745BAA81791}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1365" yWindow="2348" windowWidth="26160" windowHeight="12450" activeTab="3" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Dustin_model_rat" sheetId="10" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1524" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1524" uniqueCount="257">
   <si>
     <t>Code</t>
   </si>
@@ -790,6 +790,24 @@
   </si>
   <si>
     <t>num.blood.comp</t>
+  </si>
+  <si>
+    <t>rest of body volume fraction (slowly perfused for DCM)</t>
+  </si>
+  <si>
+    <t>tissue compartment 2 volume fraction -</t>
+  </si>
+  <si>
+    <t>tissue compartment 2 blood flow rate fraction -</t>
+  </si>
+  <si>
+    <t>rest of body blood flow rate fraction -  slowly perfused tissues</t>
+  </si>
+  <si>
+    <t>rest of body:blood partition coefficient - slowly perfused</t>
+  </si>
+  <si>
+    <t>tissue compartment 2:blood partition coefficient -</t>
   </si>
 </sst>
 </file>
@@ -1155,9 +1173,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1195,7 +1213,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1301,7 +1319,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1443,7 +1461,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1452,21 +1470,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC133E2D-914A-4425-923E-4FE379361EFA}">
   <dimension ref="A1:F104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.46875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05859375" customWidth="1"/>
+    <col min="5" max="5" width="22.29296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.29296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.52734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1486,7 +1504,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1500,7 +1518,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1511,7 +1529,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1522,7 +1540,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -1539,7 +1557,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -1556,7 +1574,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1570,7 +1588,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -1584,7 +1602,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>250</v>
       </c>
@@ -1601,7 +1619,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>159</v>
       </c>
@@ -1618,7 +1636,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>160</v>
       </c>
@@ -1635,7 +1653,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>184</v>
       </c>
@@ -1652,7 +1670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -1669,7 +1687,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>188</v>
       </c>
@@ -1686,7 +1704,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>226</v>
       </c>
@@ -1701,7 +1719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>227</v>
       </c>
@@ -1713,10 +1731,10 @@
       </c>
       <c r="E16">
         <f>SUM(E61:E75)</f>
-        <v>0.9215000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+        <v>0.92149999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1733,7 +1751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -1750,7 +1768,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>190</v>
       </c>
@@ -1767,7 +1785,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -1781,7 +1799,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>36</v>
       </c>
@@ -1795,7 +1813,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>242</v>
       </c>
@@ -1813,7 +1831,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
@@ -1827,7 +1845,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -1844,7 +1862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
@@ -1861,7 +1879,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
@@ -1872,7 +1890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>165</v>
       </c>
@@ -1887,7 +1905,7 @@
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>166</v>
       </c>
@@ -1902,7 +1920,7 @@
       </c>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
@@ -1916,7 +1934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>177</v>
       </c>
@@ -1930,7 +1948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>176</v>
       </c>
@@ -1944,7 +1962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>175</v>
       </c>
@@ -1958,7 +1976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>62</v>
       </c>
@@ -1975,7 +1993,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>63</v>
       </c>
@@ -1992,7 +2010,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>64</v>
       </c>
@@ -2009,7 +2027,7 @@
         <v>1.67</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>65</v>
       </c>
@@ -2023,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
         <v>197</v>
       </c>
@@ -2037,7 +2055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>67</v>
       </c>
@@ -2051,7 +2069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
         <v>239</v>
       </c>
@@ -2065,7 +2083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
         <v>240</v>
       </c>
@@ -2079,7 +2097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
         <v>241</v>
       </c>
@@ -2093,7 +2111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
         <v>167</v>
       </c>
@@ -2110,7 +2128,7 @@
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
         <v>168</v>
       </c>
@@ -2127,7 +2145,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
         <v>169</v>
       </c>
@@ -2144,7 +2162,7 @@
         <v>2.56</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
         <v>170</v>
       </c>
@@ -2165,7 +2183,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
         <v>171</v>
       </c>
@@ -2182,7 +2200,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
         <v>172</v>
       </c>
@@ -2203,7 +2221,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
         <v>173</v>
       </c>
@@ -2220,7 +2238,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
         <v>174</v>
       </c>
@@ -2241,7 +2259,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
         <v>48</v>
       </c>
@@ -2255,7 +2273,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
         <v>200</v>
       </c>
@@ -2266,7 +2284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A53" s="1" t="s">
         <v>50</v>
       </c>
@@ -2280,7 +2298,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
         <v>202</v>
       </c>
@@ -2294,7 +2312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
         <v>205</v>
       </c>
@@ -2308,7 +2326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
         <v>207</v>
       </c>
@@ -2319,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A57" s="1" t="s">
         <v>245</v>
       </c>
@@ -2336,7 +2354,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
         <v>52</v>
       </c>
@@ -2347,7 +2365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -2364,7 +2382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
         <v>93</v>
       </c>
@@ -2378,7 +2396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A62" s="1" t="s">
         <v>161</v>
       </c>
@@ -2392,7 +2410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A63" s="1" t="s">
         <v>162</v>
       </c>
@@ -2406,7 +2424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A64" s="1" t="s">
         <v>96</v>
       </c>
@@ -2423,7 +2441,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A65" s="1" t="s">
         <v>106</v>
       </c>
@@ -2437,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A66" s="1" t="s">
         <v>107</v>
       </c>
@@ -2454,7 +2472,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A67" s="1" t="s">
         <v>108</v>
       </c>
@@ -2468,7 +2486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A68" s="1" t="s">
         <v>109</v>
       </c>
@@ -2482,7 +2500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A69" s="1" t="s">
         <v>110</v>
       </c>
@@ -2499,12 +2517,12 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A70" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B70" t="s">
-        <v>101</v>
+        <v>252</v>
       </c>
       <c r="C70" t="s">
         <v>209</v>
@@ -2512,11 +2530,8 @@
       <c r="D70">
         <v>1</v>
       </c>
-      <c r="E70">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A71" s="1" t="s">
         <v>112</v>
       </c>
@@ -2530,7 +2545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A72" s="1" t="s">
         <v>113</v>
       </c>
@@ -2544,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A73" s="1" t="s">
         <v>114</v>
       </c>
@@ -2558,7 +2573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A74" s="1" t="s">
         <v>115</v>
       </c>
@@ -2575,12 +2590,12 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A75" s="1" t="s">
         <v>210</v>
       </c>
       <c r="B75" t="s">
-        <v>211</v>
+        <v>251</v>
       </c>
       <c r="C75" t="s">
         <v>209</v>
@@ -2588,8 +2603,11 @@
       <c r="D75">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E75">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A76" s="1" t="s">
         <v>124</v>
       </c>
@@ -2603,7 +2621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A77" s="1" t="s">
         <v>125</v>
       </c>
@@ -2620,7 +2638,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A78" s="1" t="s">
         <v>126</v>
       </c>
@@ -2634,7 +2652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A79" s="1" t="s">
         <v>127</v>
       </c>
@@ -2651,12 +2669,12 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B80" t="s">
-        <v>119</v>
+        <v>253</v>
       </c>
       <c r="C80" t="s">
         <v>204</v>
@@ -2664,11 +2682,8 @@
       <c r="D80">
         <v>0</v>
       </c>
-      <c r="E80">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A81" s="1" t="s">
         <v>129</v>
       </c>
@@ -2682,7 +2697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A82" s="1" t="s">
         <v>130</v>
       </c>
@@ -2696,7 +2711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A83" s="1" t="s">
         <v>131</v>
       </c>
@@ -2710,7 +2725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A84" s="1" t="s">
         <v>132</v>
       </c>
@@ -2727,12 +2742,12 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A85" s="1" t="s">
         <v>212</v>
       </c>
       <c r="B85" t="s">
-        <v>213</v>
+        <v>254</v>
       </c>
       <c r="C85" t="s">
         <v>204</v>
@@ -2740,8 +2755,11 @@
       <c r="D85">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E85">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A86" s="1" t="s">
         <v>144</v>
       </c>
@@ -2755,7 +2773,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A87" s="1" t="s">
         <v>145</v>
       </c>
@@ -2766,7 +2784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>146</v>
       </c>
@@ -2780,7 +2798,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A89" s="1" t="s">
         <v>147</v>
       </c>
@@ -2791,7 +2809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A90" s="1" t="s">
         <v>148</v>
       </c>
@@ -2805,21 +2823,18 @@
         <v>6.19</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A91" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B91" t="s">
-        <v>137</v>
+        <v>256</v>
       </c>
       <c r="D91">
         <v>1</v>
       </c>
-      <c r="E91">
-        <v>0.40799999999999997</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A92" s="1" t="s">
         <v>150</v>
       </c>
@@ -2830,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A93" s="1" t="s">
         <v>151</v>
       </c>
@@ -2841,7 +2856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A94" s="1" t="s">
         <v>152</v>
       </c>
@@ -2852,7 +2867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A95" s="1" t="s">
         <v>153</v>
       </c>
@@ -2866,18 +2881,21 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A96" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B96" t="s">
-        <v>215</v>
+        <v>255</v>
       </c>
       <c r="D96">
         <v>1</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E96">
+        <v>0.40799999999999997</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A98" s="1" t="s">
         <v>0</v>
       </c>
@@ -2894,7 +2912,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A99" s="1" t="s">
         <v>42</v>
       </c>
@@ -2902,7 +2920,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A101" s="1" t="s">
         <v>0</v>
       </c>
@@ -2917,7 +2935,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A102" s="1" t="s">
         <v>86</v>
       </c>
@@ -2925,7 +2943,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A103" s="1" t="s">
         <v>88</v>
       </c>
@@ -2933,7 +2951,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A104" s="1" t="s">
         <v>90</v>
       </c>
@@ -2973,21 +2991,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73575C3-523D-4B26-AB43-BBFCD1A9F157}">
   <dimension ref="A1:F104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.46875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05859375" customWidth="1"/>
+    <col min="5" max="5" width="22.29296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.29296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.52734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3007,7 +3025,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -3021,7 +3039,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -3032,7 +3050,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3043,7 +3061,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -3060,7 +3078,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -3077,7 +3095,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -3091,7 +3109,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -3105,7 +3123,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>250</v>
       </c>
@@ -3122,7 +3140,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>159</v>
       </c>
@@ -3139,7 +3157,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>160</v>
       </c>
@@ -3156,7 +3174,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>184</v>
       </c>
@@ -3173,7 +3191,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -3190,7 +3208,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>188</v>
       </c>
@@ -3207,7 +3225,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>226</v>
       </c>
@@ -3222,7 +3240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>227</v>
       </c>
@@ -3237,7 +3255,7 @@
         <v>0.92149999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -3254,7 +3272,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -3271,7 +3289,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>190</v>
       </c>
@@ -3288,7 +3306,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -3302,7 +3320,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>36</v>
       </c>
@@ -3316,7 +3334,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>242</v>
       </c>
@@ -3334,7 +3352,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
@@ -3348,7 +3366,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -3365,7 +3383,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
@@ -3382,7 +3400,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
@@ -3393,7 +3411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>165</v>
       </c>
@@ -3408,7 +3426,7 @@
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>166</v>
       </c>
@@ -3423,7 +3441,7 @@
       </c>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
@@ -3437,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>177</v>
       </c>
@@ -3451,7 +3469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>176</v>
       </c>
@@ -3465,7 +3483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>175</v>
       </c>
@@ -3479,7 +3497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>62</v>
       </c>
@@ -3496,7 +3514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>63</v>
       </c>
@@ -3513,7 +3531,7 @@
         <v>4.3099999999999996</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>64</v>
       </c>
@@ -3530,7 +3548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>65</v>
       </c>
@@ -3544,7 +3562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
         <v>197</v>
       </c>
@@ -3558,7 +3576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>67</v>
       </c>
@@ -3572,7 +3590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
         <v>239</v>
       </c>
@@ -3586,7 +3604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
         <v>240</v>
       </c>
@@ -3600,7 +3618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
         <v>241</v>
       </c>
@@ -3614,7 +3632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
         <v>167</v>
       </c>
@@ -3631,7 +3649,7 @@
         <v>9.42</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
         <v>168</v>
       </c>
@@ -3648,7 +3666,7 @@
         <v>0.433</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
         <v>169</v>
       </c>
@@ -3665,7 +3683,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
         <v>170</v>
       </c>
@@ -3686,7 +3704,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
         <v>171</v>
       </c>
@@ -3703,7 +3721,7 @@
         <v>0.433</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
         <v>172</v>
       </c>
@@ -3724,7 +3742,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
         <v>173</v>
       </c>
@@ -3741,7 +3759,7 @@
         <v>0.433</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
         <v>174</v>
       </c>
@@ -3762,7 +3780,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
         <v>48</v>
       </c>
@@ -3776,7 +3794,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
         <v>200</v>
       </c>
@@ -3787,7 +3805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A53" s="1" t="s">
         <v>50</v>
       </c>
@@ -3801,7 +3819,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
         <v>202</v>
       </c>
@@ -3815,7 +3833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
         <v>205</v>
       </c>
@@ -3829,7 +3847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
         <v>207</v>
       </c>
@@ -3840,7 +3858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A57" s="1" t="s">
         <v>245</v>
       </c>
@@ -3857,7 +3875,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
         <v>52</v>
       </c>
@@ -3868,7 +3886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -3885,7 +3903,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
         <v>93</v>
       </c>
@@ -3899,7 +3917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A62" s="1" t="s">
         <v>161</v>
       </c>
@@ -3913,7 +3931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A63" s="1" t="s">
         <v>162</v>
       </c>
@@ -3927,7 +3945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A64" s="1" t="s">
         <v>96</v>
       </c>
@@ -3944,7 +3962,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A65" s="1" t="s">
         <v>106</v>
       </c>
@@ -3958,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A66" s="1" t="s">
         <v>107</v>
       </c>
@@ -3975,7 +3993,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A67" s="1" t="s">
         <v>108</v>
       </c>
@@ -3989,7 +4007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A68" s="1" t="s">
         <v>109</v>
       </c>
@@ -4003,7 +4021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A69" s="1" t="s">
         <v>110</v>
       </c>
@@ -4020,7 +4038,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A70" s="1" t="s">
         <v>111</v>
       </c>
@@ -4037,7 +4055,7 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A71" s="1" t="s">
         <v>112</v>
       </c>
@@ -4051,7 +4069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A72" s="1" t="s">
         <v>113</v>
       </c>
@@ -4065,7 +4083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A73" s="1" t="s">
         <v>114</v>
       </c>
@@ -4079,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A74" s="1" t="s">
         <v>115</v>
       </c>
@@ -4096,7 +4114,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A75" s="1" t="s">
         <v>210</v>
       </c>
@@ -4110,7 +4128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A76" s="1" t="s">
         <v>124</v>
       </c>
@@ -4124,7 +4142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A77" s="1" t="s">
         <v>125</v>
       </c>
@@ -4141,7 +4159,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A78" s="1" t="s">
         <v>126</v>
       </c>
@@ -4155,7 +4173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A79" s="1" t="s">
         <v>127</v>
       </c>
@@ -4172,7 +4190,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>128</v>
       </c>
@@ -4189,7 +4207,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A81" s="1" t="s">
         <v>129</v>
       </c>
@@ -4203,7 +4221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A82" s="1" t="s">
         <v>130</v>
       </c>
@@ -4217,7 +4235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A83" s="1" t="s">
         <v>131</v>
       </c>
@@ -4231,7 +4249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A84" s="1" t="s">
         <v>132</v>
       </c>
@@ -4248,7 +4266,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A85" s="1" t="s">
         <v>212</v>
       </c>
@@ -4262,7 +4280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A86" s="1" t="s">
         <v>144</v>
       </c>
@@ -4276,7 +4294,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A87" s="1" t="s">
         <v>145</v>
       </c>
@@ -4287,7 +4305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>146</v>
       </c>
@@ -4301,7 +4319,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A89" s="1" t="s">
         <v>147</v>
       </c>
@@ -4312,7 +4330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A90" s="1" t="s">
         <v>148</v>
       </c>
@@ -4326,7 +4344,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A91" s="1" t="s">
         <v>149</v>
       </c>
@@ -4340,7 +4358,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A92" s="1" t="s">
         <v>150</v>
       </c>
@@ -4351,7 +4369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A93" s="1" t="s">
         <v>151</v>
       </c>
@@ -4362,7 +4380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A94" s="1" t="s">
         <v>152</v>
       </c>
@@ -4373,7 +4391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A95" s="1" t="s">
         <v>153</v>
       </c>
@@ -4387,7 +4405,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A96" s="1" t="s">
         <v>214</v>
       </c>
@@ -4398,7 +4416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A98" s="1" t="s">
         <v>0</v>
       </c>
@@ -4415,7 +4433,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A99" s="1" t="s">
         <v>42</v>
       </c>
@@ -4423,7 +4441,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A101" s="1" t="s">
         <v>0</v>
       </c>
@@ -4438,7 +4456,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A102" s="1" t="s">
         <v>86</v>
       </c>
@@ -4446,7 +4464,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A103" s="1" t="s">
         <v>88</v>
       </c>
@@ -4454,7 +4472,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A104" s="1" t="s">
         <v>90</v>
       </c>
@@ -4493,21 +4511,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDC8215B-69D8-4721-B281-D64038245121}">
   <dimension ref="A1:F102"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.46875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05859375" customWidth="1"/>
+    <col min="5" max="5" width="22.29296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.29296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.52734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4527,7 +4545,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -4541,7 +4559,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -4552,7 +4570,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -4563,7 +4581,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -4580,7 +4598,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -4597,7 +4615,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -4611,7 +4629,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -4625,7 +4643,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>250</v>
       </c>
@@ -4642,7 +4660,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>159</v>
       </c>
@@ -4659,7 +4677,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>160</v>
       </c>
@@ -4676,7 +4694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>184</v>
       </c>
@@ -4693,7 +4711,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -4710,7 +4728,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>188</v>
       </c>
@@ -4727,7 +4745,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>226</v>
       </c>
@@ -4742,7 +4760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>227</v>
       </c>
@@ -4757,7 +4775,7 @@
         <v>0.98050000000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -4774,7 +4792,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -4791,7 +4809,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
@@ -4805,7 +4823,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -4819,7 +4837,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>242</v>
       </c>
@@ -4837,7 +4855,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -4851,7 +4869,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -4868,7 +4886,7 @@
         <v>15.9</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
@@ -4879,7 +4897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>165</v>
       </c>
@@ -4894,7 +4912,7 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>166</v>
       </c>
@@ -4909,7 +4927,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
@@ -4923,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>177</v>
       </c>
@@ -4937,7 +4955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>176</v>
       </c>
@@ -4951,7 +4969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>175</v>
       </c>
@@ -4965,7 +4983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>62</v>
       </c>
@@ -4982,7 +5000,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
@@ -4999,7 +5017,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
@@ -5016,7 +5034,7 @@
         <v>1.67</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
@@ -5030,7 +5048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>197</v>
       </c>
@@ -5044,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -5058,7 +5076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
         <v>239</v>
       </c>
@@ -5072,7 +5090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>240</v>
       </c>
@@ -5086,7 +5104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
         <v>241</v>
       </c>
@@ -5100,7 +5118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
         <v>167</v>
       </c>
@@ -5117,7 +5135,7 @@
         <v>3.992</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
         <v>168</v>
       </c>
@@ -5134,7 +5152,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
         <v>169</v>
       </c>
@@ -5151,7 +5169,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
         <v>170</v>
       </c>
@@ -5172,7 +5190,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
         <v>171</v>
       </c>
@@ -5189,7 +5207,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
         <v>172</v>
       </c>
@@ -5210,7 +5228,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
         <v>173</v>
       </c>
@@ -5227,7 +5245,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
         <v>174</v>
       </c>
@@ -5248,7 +5266,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
@@ -5262,7 +5280,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
         <v>200</v>
       </c>
@@ -5273,7 +5291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -5287,7 +5305,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
         <v>202</v>
       </c>
@@ -5301,7 +5319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A53" s="1" t="s">
         <v>205</v>
       </c>
@@ -5315,7 +5333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
         <v>207</v>
       </c>
@@ -5326,7 +5344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
         <v>245</v>
       </c>
@@ -5343,7 +5361,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
         <v>52</v>
       </c>
@@ -5354,7 +5372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
         <v>0</v>
       </c>
@@ -5371,7 +5389,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A59" s="1" t="s">
         <v>93</v>
       </c>
@@ -5388,7 +5406,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
         <v>161</v>
       </c>
@@ -5402,7 +5420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
         <v>162</v>
       </c>
@@ -5416,7 +5434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A62" s="1" t="s">
         <v>96</v>
       </c>
@@ -5433,7 +5451,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A63" s="1" t="s">
         <v>106</v>
       </c>
@@ -5447,7 +5465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A64" s="1" t="s">
         <v>107</v>
       </c>
@@ -5464,7 +5482,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A65" s="1" t="s">
         <v>108</v>
       </c>
@@ -5478,7 +5496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A66" s="1" t="s">
         <v>109</v>
       </c>
@@ -5492,7 +5510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A67" s="1" t="s">
         <v>110</v>
       </c>
@@ -5509,7 +5527,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A68" s="1" t="s">
         <v>111</v>
       </c>
@@ -5526,7 +5544,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A69" s="1" t="s">
         <v>112</v>
       </c>
@@ -5540,7 +5558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A70" s="1" t="s">
         <v>113</v>
       </c>
@@ -5554,7 +5572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A71" s="1" t="s">
         <v>114</v>
       </c>
@@ -5568,7 +5586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A72" s="1" t="s">
         <v>115</v>
       </c>
@@ -5585,7 +5603,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A73" s="1" t="s">
         <v>210</v>
       </c>
@@ -5599,7 +5617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A74" s="1" t="s">
         <v>124</v>
       </c>
@@ -5613,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A75" s="1" t="s">
         <v>125</v>
       </c>
@@ -5630,7 +5648,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A76" s="1" t="s">
         <v>126</v>
       </c>
@@ -5644,7 +5662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A77" s="1" t="s">
         <v>127</v>
       </c>
@@ -5661,7 +5679,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A78" s="1" t="s">
         <v>128</v>
       </c>
@@ -5678,7 +5696,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A79" s="1" t="s">
         <v>129</v>
       </c>
@@ -5692,7 +5710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>130</v>
       </c>
@@ -5706,7 +5724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A81" s="1" t="s">
         <v>131</v>
       </c>
@@ -5720,7 +5738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A82" s="1" t="s">
         <v>132</v>
       </c>
@@ -5737,7 +5755,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A83" s="1" t="s">
         <v>212</v>
       </c>
@@ -5751,7 +5769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A84" s="1" t="s">
         <v>144</v>
       </c>
@@ -5765,7 +5783,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A85" s="1" t="s">
         <v>145</v>
       </c>
@@ -5776,7 +5794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A86" s="1" t="s">
         <v>146</v>
       </c>
@@ -5790,7 +5808,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A87" s="1" t="s">
         <v>147</v>
       </c>
@@ -5801,7 +5819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>148</v>
       </c>
@@ -5815,7 +5833,7 @@
         <v>6.19</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A89" s="1" t="s">
         <v>149</v>
       </c>
@@ -5829,7 +5847,7 @@
         <v>0.40799999999999997</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A90" s="1" t="s">
         <v>150</v>
       </c>
@@ -5840,7 +5858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A91" s="1" t="s">
         <v>151</v>
       </c>
@@ -5851,7 +5869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A92" s="1" t="s">
         <v>152</v>
       </c>
@@ -5862,7 +5880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A93" s="1" t="s">
         <v>153</v>
       </c>
@@ -5876,7 +5894,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A94" s="1" t="s">
         <v>214</v>
       </c>
@@ -5887,7 +5905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A96" s="1" t="s">
         <v>0</v>
       </c>
@@ -5904,7 +5922,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A97" s="1" t="s">
         <v>42</v>
       </c>
@@ -5912,7 +5930,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A99" s="1" t="s">
         <v>0</v>
       </c>
@@ -5927,7 +5945,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A100" s="1" t="s">
         <v>86</v>
       </c>
@@ -5935,7 +5953,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A101" s="1" t="s">
         <v>88</v>
       </c>
@@ -5943,7 +5961,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A102" s="1" t="s">
         <v>90</v>
       </c>
@@ -5982,21 +6000,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C669BE20-7CF4-4C3C-8BC2-1F87982D51B2}">
   <dimension ref="A1:F102"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.46875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05859375" customWidth="1"/>
+    <col min="5" max="5" width="22.29296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.29296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.52734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6016,7 +6034,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -6030,7 +6048,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -6041,7 +6059,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -6052,7 +6070,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -6069,7 +6087,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -6086,7 +6104,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -6100,7 +6118,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -6114,7 +6132,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>250</v>
       </c>
@@ -6131,7 +6149,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>159</v>
       </c>
@@ -6148,7 +6166,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>160</v>
       </c>
@@ -6165,7 +6183,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>184</v>
       </c>
@@ -6182,7 +6200,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -6199,7 +6217,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>188</v>
       </c>
@@ -6216,7 +6234,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>226</v>
       </c>
@@ -6231,7 +6249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>227</v>
       </c>
@@ -6243,10 +6261,10 @@
       </c>
       <c r="E16">
         <f>SUM(E59:E73)</f>
-        <v>0.9215000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+        <v>0.92149999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -6263,7 +6281,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -6280,7 +6298,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
@@ -6294,7 +6312,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -6308,7 +6326,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>242</v>
       </c>
@@ -6326,7 +6344,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -6340,7 +6358,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -6357,7 +6375,7 @@
         <v>15.9</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
@@ -6368,7 +6386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>165</v>
       </c>
@@ -6383,7 +6401,7 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>166</v>
       </c>
@@ -6398,7 +6416,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
@@ -6412,7 +6430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>177</v>
       </c>
@@ -6426,7 +6444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>176</v>
       </c>
@@ -6440,7 +6458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>175</v>
       </c>
@@ -6454,7 +6472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>62</v>
       </c>
@@ -6468,7 +6486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
@@ -6485,7 +6503,7 @@
         <v>4.3099999999999996</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
@@ -6499,7 +6517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
@@ -6513,7 +6531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>197</v>
       </c>
@@ -6527,7 +6545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -6541,7 +6559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
         <v>239</v>
       </c>
@@ -6555,7 +6573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>240</v>
       </c>
@@ -6569,7 +6587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
         <v>241</v>
       </c>
@@ -6583,7 +6601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
         <v>167</v>
       </c>
@@ -6600,7 +6618,7 @@
         <v>3.97</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
         <v>168</v>
       </c>
@@ -6617,7 +6635,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
         <v>169</v>
       </c>
@@ -6634,7 +6652,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
         <v>170</v>
       </c>
@@ -6655,7 +6673,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
         <v>171</v>
       </c>
@@ -6673,7 +6691,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
         <v>172</v>
       </c>
@@ -6694,7 +6712,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
         <v>173</v>
       </c>
@@ -6712,7 +6730,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
         <v>174</v>
       </c>
@@ -6733,7 +6751,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
@@ -6747,7 +6765,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
         <v>200</v>
       </c>
@@ -6758,7 +6776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -6772,7 +6790,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
         <v>202</v>
       </c>
@@ -6786,7 +6804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A53" s="1" t="s">
         <v>205</v>
       </c>
@@ -6800,7 +6818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
         <v>207</v>
       </c>
@@ -6811,7 +6829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
         <v>245</v>
       </c>
@@ -6828,7 +6846,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
         <v>52</v>
       </c>
@@ -6839,7 +6857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
         <v>0</v>
       </c>
@@ -6856,7 +6874,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A59" s="1" t="s">
         <v>93</v>
       </c>
@@ -6870,7 +6888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
         <v>161</v>
       </c>
@@ -6884,7 +6902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
         <v>162</v>
       </c>
@@ -6898,7 +6916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A62" s="1" t="s">
         <v>96</v>
       </c>
@@ -6915,7 +6933,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A63" s="1" t="s">
         <v>106</v>
       </c>
@@ -6929,7 +6947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A64" s="1" t="s">
         <v>107</v>
       </c>
@@ -6946,7 +6964,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A65" s="1" t="s">
         <v>108</v>
       </c>
@@ -6960,7 +6978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A66" s="1" t="s">
         <v>109</v>
       </c>
@@ -6974,7 +6992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A67" s="1" t="s">
         <v>110</v>
       </c>
@@ -6991,12 +7009,12 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A68" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B68" t="s">
-        <v>101</v>
+        <v>252</v>
       </c>
       <c r="C68" t="s">
         <v>209</v>
@@ -7004,11 +7022,8 @@
       <c r="D68">
         <v>1</v>
       </c>
-      <c r="E68">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A69" s="1" t="s">
         <v>112</v>
       </c>
@@ -7022,7 +7037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A70" s="1" t="s">
         <v>113</v>
       </c>
@@ -7036,7 +7051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A71" s="1" t="s">
         <v>114</v>
       </c>
@@ -7050,7 +7065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A72" s="1" t="s">
         <v>115</v>
       </c>
@@ -7067,12 +7082,12 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A73" s="1" t="s">
         <v>210</v>
       </c>
       <c r="B73" t="s">
-        <v>211</v>
+        <v>251</v>
       </c>
       <c r="C73" t="s">
         <v>209</v>
@@ -7080,8 +7095,11 @@
       <c r="D73">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E73">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A74" s="1" t="s">
         <v>124</v>
       </c>
@@ -7095,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A75" s="1" t="s">
         <v>125</v>
       </c>
@@ -7112,7 +7130,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A76" s="1" t="s">
         <v>126</v>
       </c>
@@ -7126,7 +7144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A77" s="1" t="s">
         <v>127</v>
       </c>
@@ -7143,12 +7161,12 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A78" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B78" t="s">
-        <v>119</v>
+        <v>253</v>
       </c>
       <c r="C78" t="s">
         <v>204</v>
@@ -7156,11 +7174,8 @@
       <c r="D78">
         <v>0</v>
       </c>
-      <c r="E78">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A79" s="1" t="s">
         <v>129</v>
       </c>
@@ -7174,7 +7189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>130</v>
       </c>
@@ -7188,7 +7203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A81" s="1" t="s">
         <v>131</v>
       </c>
@@ -7202,7 +7217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A82" s="1" t="s">
         <v>132</v>
       </c>
@@ -7219,12 +7234,12 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A83" s="1" t="s">
         <v>212</v>
       </c>
       <c r="B83" t="s">
-        <v>213</v>
+        <v>254</v>
       </c>
       <c r="C83" t="s">
         <v>204</v>
@@ -7232,8 +7247,11 @@
       <c r="D83">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E83">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A84" s="1" t="s">
         <v>144</v>
       </c>
@@ -7244,10 +7262,10 @@
         <v>1</v>
       </c>
       <c r="E84">
-        <v>0.46</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+        <v>0.73199999999999998</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A85" s="1" t="s">
         <v>145</v>
       </c>
@@ -7258,7 +7276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A86" s="1" t="s">
         <v>146</v>
       </c>
@@ -7272,7 +7290,7 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A87" s="1" t="s">
         <v>147</v>
       </c>
@@ -7283,7 +7301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>148</v>
       </c>
@@ -7297,21 +7315,18 @@
         <v>6.19</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A89" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B89" t="s">
-        <v>137</v>
+        <v>256</v>
       </c>
       <c r="D89">
         <v>1</v>
       </c>
-      <c r="E89">
-        <v>0.40799999999999997</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A90" s="1" t="s">
         <v>150</v>
       </c>
@@ -7322,7 +7337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A91" s="1" t="s">
         <v>151</v>
       </c>
@@ -7333,7 +7348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A92" s="1" t="s">
         <v>152</v>
       </c>
@@ -7344,7 +7359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A93" s="1" t="s">
         <v>153</v>
       </c>
@@ -7358,18 +7373,21 @@
         <v>0.73199999999999998</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A94" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B94" t="s">
-        <v>215</v>
+        <v>255</v>
       </c>
       <c r="D94">
         <v>1</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E94">
+        <v>0.40799999999999997</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A96" s="1" t="s">
         <v>0</v>
       </c>
@@ -7386,7 +7404,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A97" s="1" t="s">
         <v>42</v>
       </c>
@@ -7394,7 +7412,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A99" s="1" t="s">
         <v>0</v>
       </c>
@@ -7409,7 +7427,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A100" s="1" t="s">
         <v>86</v>
       </c>
@@ -7417,7 +7435,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A101" s="1" t="s">
         <v>88</v>
       </c>
@@ -7425,7 +7443,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A102" s="1" t="s">
         <v>90</v>
       </c>
@@ -7464,21 +7482,21 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED28972A-92DF-4C4A-9B3E-1FD1ED840ACF}">
   <dimension ref="A1:F102"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.46875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05859375" customWidth="1"/>
+    <col min="5" max="5" width="22.29296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.29296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.52734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.52734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7498,7 +7516,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -7512,7 +7530,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -7523,7 +7541,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -7534,7 +7552,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -7551,7 +7569,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -7568,7 +7586,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -7582,7 +7600,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -7596,7 +7614,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>250</v>
       </c>
@@ -7613,7 +7631,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>159</v>
       </c>
@@ -7630,7 +7648,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>160</v>
       </c>
@@ -7647,7 +7665,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>184</v>
       </c>
@@ -7664,7 +7682,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -7681,7 +7699,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>188</v>
       </c>
@@ -7698,7 +7716,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>226</v>
       </c>
@@ -7713,7 +7731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>227</v>
       </c>
@@ -7728,7 +7746,7 @@
         <v>0.98050000000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -7745,7 +7763,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -7762,7 +7780,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
@@ -7776,7 +7794,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -7790,7 +7808,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>242</v>
       </c>
@@ -7808,7 +7826,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -7822,7 +7840,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -7839,7 +7857,7 @@
         <v>24.2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
@@ -7850,7 +7868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>165</v>
       </c>
@@ -7865,7 +7883,7 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>166</v>
       </c>
@@ -7880,7 +7898,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
@@ -7894,7 +7912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>177</v>
       </c>
@@ -7908,7 +7926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>176</v>
       </c>
@@ -7922,7 +7940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>175</v>
       </c>
@@ -7936,7 +7954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>62</v>
       </c>
@@ -7950,7 +7968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
@@ -7967,7 +7985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
@@ -7981,7 +7999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
@@ -7995,7 +8013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>197</v>
       </c>
@@ -8009,7 +8027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -8023,7 +8041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
         <v>239</v>
       </c>
@@ -8037,7 +8055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>240</v>
       </c>
@@ -8051,7 +8069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
         <v>241</v>
       </c>
@@ -8065,7 +8083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
         <v>167</v>
       </c>
@@ -8082,7 +8100,7 @@
         <v>9.27</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
         <v>168</v>
       </c>
@@ -8099,7 +8117,7 @@
         <v>0.57399999999999995</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
         <v>169</v>
       </c>
@@ -8116,7 +8134,7 @@
         <v>1.41</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
         <v>170</v>
       </c>
@@ -8137,7 +8155,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
         <v>171</v>
       </c>
@@ -8154,7 +8172,7 @@
         <v>0.57399999999999995</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
         <v>172</v>
       </c>
@@ -8175,7 +8193,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
         <v>173</v>
       </c>
@@ -8192,7 +8210,7 @@
         <v>0.57399999999999995</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
         <v>174</v>
       </c>
@@ -8213,7 +8231,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
@@ -8227,7 +8245,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A50" s="1" t="s">
         <v>200</v>
       </c>
@@ -8238,7 +8256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -8252,7 +8270,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A52" s="1" t="s">
         <v>202</v>
       </c>
@@ -8266,7 +8284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A53" s="1" t="s">
         <v>205</v>
       </c>
@@ -8280,7 +8298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A54" s="1" t="s">
         <v>207</v>
       </c>
@@ -8291,7 +8309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A55" s="1" t="s">
         <v>245</v>
       </c>
@@ -8308,7 +8326,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A56" s="1" t="s">
         <v>52</v>
       </c>
@@ -8319,7 +8337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A58" s="1" t="s">
         <v>0</v>
       </c>
@@ -8336,7 +8354,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A59" s="1" t="s">
         <v>93</v>
       </c>
@@ -8353,7 +8371,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A60" s="1" t="s">
         <v>161</v>
       </c>
@@ -8367,7 +8385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A61" s="1" t="s">
         <v>162</v>
       </c>
@@ -8381,7 +8399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A62" s="1" t="s">
         <v>96</v>
       </c>
@@ -8398,7 +8416,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A63" s="1" t="s">
         <v>106</v>
       </c>
@@ -8412,7 +8430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A64" s="1" t="s">
         <v>107</v>
       </c>
@@ -8429,7 +8447,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A65" s="1" t="s">
         <v>108</v>
       </c>
@@ -8443,7 +8461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A66" s="1" t="s">
         <v>109</v>
       </c>
@@ -8457,7 +8475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A67" s="1" t="s">
         <v>110</v>
       </c>
@@ -8474,7 +8492,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A68" s="1" t="s">
         <v>111</v>
       </c>
@@ -8491,7 +8509,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A69" s="1" t="s">
         <v>112</v>
       </c>
@@ -8505,7 +8523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A70" s="1" t="s">
         <v>113</v>
       </c>
@@ -8519,7 +8537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A71" s="1" t="s">
         <v>114</v>
       </c>
@@ -8533,7 +8551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A72" s="1" t="s">
         <v>115</v>
       </c>
@@ -8550,7 +8568,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A73" s="1" t="s">
         <v>210</v>
       </c>
@@ -8564,7 +8582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A74" s="1" t="s">
         <v>124</v>
       </c>
@@ -8578,7 +8596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A75" s="1" t="s">
         <v>125</v>
       </c>
@@ -8595,7 +8613,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A76" s="1" t="s">
         <v>126</v>
       </c>
@@ -8609,7 +8627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A77" s="1" t="s">
         <v>127</v>
       </c>
@@ -8626,7 +8644,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A78" s="1" t="s">
         <v>128</v>
       </c>
@@ -8643,7 +8661,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A79" s="1" t="s">
         <v>129</v>
       </c>
@@ -8657,7 +8675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A80" s="1" t="s">
         <v>130</v>
       </c>
@@ -8671,7 +8689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A81" s="1" t="s">
         <v>131</v>
       </c>
@@ -8685,7 +8703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A82" s="1" t="s">
         <v>132</v>
       </c>
@@ -8702,7 +8720,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A83" s="1" t="s">
         <v>212</v>
       </c>
@@ -8716,7 +8734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A84" s="1" t="s">
         <v>144</v>
       </c>
@@ -8730,7 +8748,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A85" s="1" t="s">
         <v>145</v>
       </c>
@@ -8741,7 +8759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A86" s="1" t="s">
         <v>146</v>
       </c>
@@ -8755,7 +8773,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A87" s="1" t="s">
         <v>147</v>
       </c>
@@ -8766,7 +8784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A88" s="1" t="s">
         <v>148</v>
       </c>
@@ -8780,7 +8798,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A89" s="1" t="s">
         <v>149</v>
       </c>
@@ -8794,7 +8812,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A90" s="1" t="s">
         <v>150</v>
       </c>
@@ -8805,7 +8823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A91" s="1" t="s">
         <v>151</v>
       </c>
@@ -8816,7 +8834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A92" s="1" t="s">
         <v>152</v>
       </c>
@@ -8827,7 +8845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A93" s="1" t="s">
         <v>153</v>
       </c>
@@ -8841,7 +8859,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A94" s="1" t="s">
         <v>214</v>
       </c>
@@ -8852,7 +8870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A96" s="1" t="s">
         <v>0</v>
       </c>
@@ -8869,7 +8887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A97" s="1" t="s">
         <v>42</v>
       </c>
@@ -8877,7 +8895,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A99" s="1" t="s">
         <v>0</v>
       </c>
@@ -8892,7 +8910,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A100" s="1" t="s">
         <v>86</v>
       </c>
@@ -8900,7 +8918,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A101" s="1" t="s">
         <v>88</v>
       </c>
@@ -8908,7 +8926,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A102" s="1" t="s">
         <v>90</v>
       </c>
@@ -8945,51 +8963,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -9462,12 +9435,12 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -9476,7 +9449,91 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7345DC6-CAC3-4709-BA76-1291BF3A473B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9486,26 +9543,7 @@
     <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7345DC6-CAC3-4709-BA76-1291BF3A473B}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>